<commit_message>
Some file name changes
</commit_message>
<xml_diff>
--- a/data/prod_parameters/MachineryAndEnergyMgmt.xlsx
+++ b/data/prod_parameters/MachineryAndEnergyMgmt.xlsx
@@ -249,9 +249,6 @@
     <t>Flytgödsel</t>
   </si>
   <si>
-    <t>MachineryAndEnergyMgmt_field_operations.csv</t>
-  </si>
-  <si>
     <t>field_operations</t>
   </si>
   <si>
@@ -659,6 +656,9 @@
   </si>
   <si>
     <t>biodiesel</t>
+  </si>
+  <si>
+    <t>MachineryAndEnergyMgmt-field_operations.csv</t>
   </si>
 </sst>
 </file>
@@ -1126,22 +1126,22 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B1" s="14" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E1" s="14" t="s">
         <v>44</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G1" s="14" t="s">
         <v>1</v>
@@ -1161,92 +1161,92 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G2" s="20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H2" s="9">
         <v>0</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J2" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H4" s="18">
         <f>(241822577+237201100)/(241822577+237201100+5856000+8368914)*100</f>
         <v>97.116076100458642</v>
       </c>
       <c r="I4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H5" s="18">
         <f>100-H4</f>
         <v>2.8839238995413581</v>
       </c>
       <c r="I5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H6" s="10">
         <v>0</v>
       </c>
       <c r="I6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H7" s="10">
         <v>0</v>
       </c>
       <c r="I7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -1256,161 +1256,161 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>159</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="G9" s="6" t="s">
         <v>160</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>161</v>
       </c>
       <c r="H9" s="11">
         <v>6.4777062142923141</v>
       </c>
       <c r="I9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>159</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="G10" s="6" t="s">
         <v>160</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>161</v>
       </c>
       <c r="H10" s="11">
         <v>8.7567853491111922</v>
       </c>
       <c r="I10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K10" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>159</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="G11" s="6" t="s">
         <v>160</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>161</v>
       </c>
       <c r="H11" s="18">
         <v>59.671114354829328</v>
       </c>
       <c r="I11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J11" s="19" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="K11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>159</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="G12" s="6" t="s">
         <v>160</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>161</v>
       </c>
       <c r="H12" s="18">
         <v>16.802918820320372</v>
       </c>
       <c r="I12" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>159</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="G13" s="6" t="s">
         <v>160</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>161</v>
       </c>
       <c r="H13" s="11">
         <v>7.4851294970113242</v>
       </c>
       <c r="I13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>159</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="G14" s="6" t="s">
         <v>160</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>158</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>161</v>
       </c>
       <c r="H14" s="11">
         <v>0.80634576443547301</v>
       </c>
       <c r="I14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F16" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G16" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H16" s="15">
         <v>80</v>
       </c>
       <c r="I16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F17" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G17" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H17" s="15">
         <v>10</v>
       </c>
       <c r="I17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F18" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G18" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H18" s="15">
         <v>10</v>
       </c>
       <c r="I18" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -1488,13 +1488,13 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H24">
         <v>2</v>
       </c>
       <c r="I24" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J24" s="7"/>
     </row>
@@ -1562,14 +1562,14 @@
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
       <c r="G28" s="20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H28" s="9">
         <v>1</v>
       </c>
       <c r="I28" s="9"/>
       <c r="J28" s="21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="18" x14ac:dyDescent="0.35">
@@ -1581,67 +1581,67 @@
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
       <c r="G29" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H29">
         <v>0.26</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B30" s="4"/>
       <c r="C30" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
       <c r="G30" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H30">
         <v>0.26</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B31" s="4"/>
       <c r="C31" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
       <c r="G31" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H31">
         <v>0.45</v>
       </c>
       <c r="J31" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B32" s="4"/>
       <c r="C32" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
       <c r="F32" s="6"/>
       <c r="G32" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H32">
         <v>0.76</v>
       </c>
       <c r="J32" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
@@ -1680,7 +1680,7 @@
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G36" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H36">
         <v>4</v>
@@ -1794,123 +1794,123 @@
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G46" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H46" s="9">
         <v>0</v>
       </c>
       <c r="I46" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J46" s="9"/>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G47" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H47" s="9">
         <v>0</v>
       </c>
       <c r="I47" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J47" s="9"/>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G48" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H48" s="9">
         <v>0</v>
       </c>
       <c r="I48" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J48" s="9"/>
     </row>
     <row r="49" spans="4:11" x14ac:dyDescent="0.25">
       <c r="G49" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H49" s="9">
         <v>0</v>
       </c>
       <c r="I49" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="J49" s="9"/>
     </row>
     <row r="50" spans="4:11" x14ac:dyDescent="0.25">
       <c r="G50" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H50" s="9">
         <v>0</v>
       </c>
       <c r="I50" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J50" s="9"/>
     </row>
     <row r="51" spans="4:11" x14ac:dyDescent="0.25">
       <c r="G51" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H51" s="9">
         <v>1</v>
       </c>
       <c r="I51" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J51" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="52" spans="4:11" x14ac:dyDescent="0.25">
       <c r="G52" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H52" s="9">
         <v>0</v>
       </c>
       <c r="I52" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J52" s="9"/>
     </row>
     <row r="53" spans="4:11" x14ac:dyDescent="0.25">
       <c r="G53" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H53" s="9">
         <v>0</v>
       </c>
       <c r="I53" s="9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J53" s="9"/>
     </row>
     <row r="54" spans="4:11" x14ac:dyDescent="0.25">
       <c r="G54" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H54" s="9">
         <v>0</v>
       </c>
       <c r="I54" s="9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J54" s="9"/>
     </row>
     <row r="55" spans="4:11" x14ac:dyDescent="0.25">
       <c r="G55" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H55" s="9">
         <v>0</v>
       </c>
       <c r="I55" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J55" s="9"/>
     </row>
@@ -1922,26 +1922,26 @@
     </row>
     <row r="57" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D57" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G57" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H57" s="10">
         <v>364</v>
       </c>
       <c r="I57" s="10"/>
       <c r="J57" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K57" s="10"/>
     </row>
     <row r="58" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D58" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G58" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H58" s="10">
         <v>18.8</v>
@@ -1952,10 +1952,10 @@
     </row>
     <row r="59" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D59" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G59" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H59" s="10">
         <v>0</v>
@@ -1966,10 +1966,10 @@
     </row>
     <row r="60" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D60" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G60" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H60" s="10">
         <v>10</v>
@@ -1980,13 +1980,13 @@
     </row>
     <row r="61" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D61" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E61" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G61" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H61" s="12">
         <v>1</v>
@@ -1997,13 +1997,13 @@
     </row>
     <row r="62" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D62" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E62" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G62" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H62" s="10">
         <v>0.88</v>
@@ -2014,13 +2014,13 @@
     </row>
     <row r="63" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D63" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E63" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G63" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H63" s="10">
         <v>0.78</v>
@@ -2038,26 +2038,26 @@
     </row>
     <row r="65" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D65" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G65" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H65" s="10">
         <v>652</v>
       </c>
       <c r="I65" s="10"/>
       <c r="J65" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="K65" s="10"/>
     </row>
     <row r="66" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D66" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G66" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H66" s="10">
         <v>0</v>
@@ -2068,10 +2068,10 @@
     </row>
     <row r="67" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D67" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G67" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H67" s="10">
         <v>5.0999999999999996</v>
@@ -2082,10 +2082,10 @@
     </row>
     <row r="68" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D68" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G68" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H68" s="10">
         <v>20</v>
@@ -2096,13 +2096,13 @@
     </row>
     <row r="69" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D69" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E69" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G69" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H69" s="12">
         <v>1</v>
@@ -2113,13 +2113,13 @@
     </row>
     <row r="70" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D70" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E70" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G70" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H70" s="12">
         <v>0.7</v>
@@ -2130,13 +2130,13 @@
     </row>
     <row r="71" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D71" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E71" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G71" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H71" s="10">
         <v>0.45</v>
@@ -2154,26 +2154,26 @@
     </row>
     <row r="73" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D73" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G73" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H73" s="10">
         <v>46</v>
       </c>
       <c r="I73" s="10"/>
       <c r="J73" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K73" s="10"/>
     </row>
     <row r="74" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D74" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G74" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H74" s="10">
         <v>2.8</v>
@@ -2184,10 +2184,10 @@
     </row>
     <row r="75" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D75" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G75" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H75" s="10">
         <v>0</v>
@@ -2198,10 +2198,10 @@
     </row>
     <row r="76" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D76" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G76" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H76" s="10">
         <v>5</v>
@@ -2212,13 +2212,13 @@
     </row>
     <row r="77" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D77" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E77" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G77" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H77" s="12">
         <v>1</v>
@@ -2229,13 +2229,13 @@
     </row>
     <row r="78" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D78" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E78" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G78" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H78" s="10">
         <v>0.85</v>
@@ -2246,13 +2246,13 @@
     </row>
     <row r="79" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D79" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E79" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G79" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H79" s="10">
         <v>0.65</v>
@@ -2270,38 +2270,38 @@
     </row>
     <row r="81" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D81" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G81" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H81" s="12">
         <v>5.0999999999999996</v>
       </c>
       <c r="I81" s="10"/>
       <c r="J81" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="K81" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="82" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D82" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G82" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H82" s="12">
         <v>7.1</v>
       </c>
       <c r="I82" s="10"/>
       <c r="J82" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K82" s="4" t="s">
         <v>96</v>
-      </c>
-      <c r="K82" s="4" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="83" spans="2:11" x14ac:dyDescent="0.25">
@@ -2313,46 +2313,46 @@
     </row>
     <row r="84" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D84" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G84" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H84" s="12">
         <v>3.7353333333333332</v>
       </c>
       <c r="I84" s="10"/>
       <c r="J84" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="K84" s="6" t="s">
         <v>89</v>
-      </c>
-      <c r="K84" s="6" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="85" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D85" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G85" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H85" s="11">
         <v>17.096931944444446</v>
       </c>
       <c r="I85" s="10"/>
       <c r="J85" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="K85" s="4" t="s">
         <v>91</v>
-      </c>
-      <c r="K85" s="4" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="86" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D86" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G86" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H86" s="12">
         <v>1.2451111111111113</v>
@@ -2362,15 +2362,15 @@
         <v>47</v>
       </c>
       <c r="K86" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="87" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D87" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G87" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H87" s="12">
         <v>3.1127777777777781</v>
@@ -2380,233 +2380,233 @@
         <v>48</v>
       </c>
       <c r="K87" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="88" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D88" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G88" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H88" s="12">
         <v>4.6691666666666665</v>
       </c>
       <c r="I88" s="10"/>
       <c r="J88" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K88" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="89" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D89" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G89" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H89" s="12">
         <v>3.1127777777777781</v>
       </c>
       <c r="I89" s="10"/>
       <c r="J89" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K89" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="90" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D90" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G90" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H90" s="11">
         <v>11.828555555555555</v>
       </c>
       <c r="I90" s="10"/>
       <c r="J90" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="K90" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="91" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D91" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G91" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H91" s="11">
         <v>26.302972222222223</v>
       </c>
       <c r="I91" s="10"/>
       <c r="J91" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K91" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="92" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D92" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G92" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H92" s="11">
         <v>11.3</v>
       </c>
       <c r="I92" s="10"/>
       <c r="J92" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="K92" s="10" t="s">
         <v>107</v>
-      </c>
-      <c r="K92" s="10" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="93" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D93" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G93" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H93" s="11">
         <v>23.278130416666666</v>
       </c>
       <c r="I93" s="10"/>
       <c r="J93" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K93" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="94" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D94" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G94" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H94" s="10">
         <v>13.15</v>
       </c>
       <c r="I94" s="10"/>
       <c r="J94" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K94" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="95" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D95" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G95" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H95" s="10">
         <v>5.26</v>
       </c>
       <c r="I95" s="10"/>
       <c r="J95" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K95" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="96" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B96" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D96" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G96" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H96" s="12">
         <v>1.7546281240590185</v>
       </c>
       <c r="I96" s="10"/>
       <c r="J96" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="K96" s="4" t="s">
         <v>112</v>
-      </c>
-      <c r="K96" s="4" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B97" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D97" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G97" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H97" s="12">
         <v>5.1828516694033944</v>
       </c>
       <c r="I97" s="10"/>
       <c r="J97" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="K97" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B98" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D98" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G98" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H98" s="13">
         <v>4.0531064740502947</v>
       </c>
       <c r="J98" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K98" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B99" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D99" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G99" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H99" s="13">
         <v>4.3591310772039646</v>
       </c>
       <c r="J99" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K99" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.25">
@@ -2617,71 +2617,71 @@
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D101" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G101" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H101" s="13">
         <v>14.6</v>
       </c>
       <c r="J101" s="6"/>
       <c r="K101" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D102" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F102" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G102" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H102" s="13">
         <v>37.744765138888887</v>
       </c>
       <c r="J102" s="6"/>
       <c r="K102" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D103" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F103" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G103" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H103" s="13">
         <v>50.107162083333336</v>
       </c>
       <c r="J103" s="6"/>
       <c r="K103" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D104" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F104" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G104" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H104" s="13">
         <v>36.955675972222224</v>
       </c>
       <c r="J104" s="6"/>
       <c r="K104" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.25">
@@ -2692,58 +2692,58 @@
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D106" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G106" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H106" s="13">
         <v>1.6176327916666666</v>
       </c>
       <c r="J106" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K106" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D107" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G107" s="10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H107" s="13">
         <v>3.0774477499999997</v>
       </c>
       <c r="J107" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="K107" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D108" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G108" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H108" s="13">
         <v>0.25</v>
       </c>
       <c r="J108" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K108" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
@@ -2758,26 +2758,26 @@
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G111" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H111" s="9">
         <v>0</v>
       </c>
       <c r="J111" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G112" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H112" t="s">
-        <v>49</v>
+        <v>181</v>
       </c>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B114" s="1"/>
       <c r="C114" s="1"/>
@@ -2792,144 +2792,144 @@
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G115" s="9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H115" s="9">
         <v>0</v>
       </c>
       <c r="I115" s="9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="J115" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B116" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G116" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H116">
         <v>302</v>
       </c>
       <c r="I116" t="s">
+        <v>169</v>
+      </c>
+      <c r="J116" t="s">
         <v>170</v>
       </c>
-      <c r="J116" t="s">
-        <v>171</v>
-      </c>
       <c r="K116" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B117" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G117" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H117">
         <v>197</v>
       </c>
       <c r="I117" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="J117" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K117" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B118" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G118" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H118">
         <v>216</v>
       </c>
       <c r="I118" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="J118" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="K118" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B119" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G119" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H119">
         <v>216</v>
       </c>
       <c r="I119" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="J119" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B120" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G120" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H120">
         <v>216</v>
       </c>
       <c r="I120" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="J120" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B121" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G121" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H121">
         <v>216</v>
       </c>
       <c r="I121" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="J121" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B122" t="s">
+        <v>167</v>
+      </c>
+      <c r="G122" t="s">
         <v>168</v>
-      </c>
-      <c r="G122" t="s">
-        <v>169</v>
       </c>
       <c r="H122">
         <v>216</v>
       </c>
       <c r="I122" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="J122" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -2945,52 +2945,52 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implemented calculation of energy use emissions
</commit_message>
<xml_diff>
--- a/data/prod_parameters/MachineryAndEnergyMgmt.xlsx
+++ b/data/prod_parameters/MachineryAndEnergyMgmt.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="10650"/>
   </bookViews>
   <sheets>
     <sheet name="default" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="201">
   <si>
     <t>f_crop</t>
   </si>
@@ -660,15 +660,85 @@
   <si>
     <t>MachineryAndEnergyMgmt-field_operations.csv</t>
   </si>
+  <si>
+    <t>f_compound</t>
+  </si>
+  <si>
+    <t>combustion_EF</t>
+  </si>
+  <si>
+    <t>CO2</t>
+  </si>
+  <si>
+    <t>N2O</t>
+  </si>
+  <si>
+    <r>
+      <t>Fuel combustion emission factors</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (add non-GHG compunds?)</t>
+    </r>
+  </si>
+  <si>
+    <t>IPCC Guidelines 2006. Chapter 3, Table 3.2.1</t>
+  </si>
+  <si>
+    <t>Gas/ Diesel Oil</t>
+  </si>
+  <si>
+    <t>IPCC Guidelines 2006. Chapter 3, Table 3.2.2</t>
+  </si>
+  <si>
+    <t>assume same as diesel</t>
+  </si>
+  <si>
+    <t>no emissions?</t>
+  </si>
+  <si>
+    <t>CH4fos</t>
+  </si>
+  <si>
+    <t>CH4bio</t>
+  </si>
+  <si>
+    <t>kg/TJ</t>
+  </si>
+  <si>
+    <t>Wood / Wood Waste</t>
+  </si>
+  <si>
+    <t>Natural Gas</t>
+  </si>
+  <si>
+    <t>Crude Oil</t>
+  </si>
+  <si>
+    <t>IPCC Guidelines 2006. Chapter 2, Table 2.5</t>
+  </si>
+  <si>
+    <t>grain drying</t>
+  </si>
+  <si>
+    <t>Fallback</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="168" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -740,6 +810,13 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="2" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -810,7 +887,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -833,6 +910,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1113,18 +1195,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O122"/>
+  <dimension ref="A1:P148"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="6" width="12.28515625" customWidth="1"/>
-    <col min="7" max="7" width="31" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.28515625" customWidth="1"/>
-    <col min="9" max="9" width="12.140625" customWidth="1"/>
-    <col min="10" max="10" width="31.7109375" customWidth="1"/>
-    <col min="11" max="11" width="22.7109375" customWidth="1"/>
+    <col min="3" max="7" width="12.28515625" customWidth="1"/>
+    <col min="8" max="8" width="31" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.28515625" customWidth="1"/>
+    <col min="10" max="10" width="12.140625" customWidth="1"/>
+    <col min="11" max="11" width="31.7109375" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>152</v>
       </c>
@@ -1144,1791 +1226,2326 @@
         <v>129</v>
       </c>
       <c r="G1" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="H1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="I1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="14" t="s">
+      <c r="J1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="14" t="s">
+      <c r="K1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="14" t="s">
+      <c r="L1" s="14" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="G2" s="20" t="s">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H2" s="20" t="s">
         <v>160</v>
       </c>
-      <c r="H2" s="9">
+      <c r="I2" s="9">
         <v>0</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="J2" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="K2" s="9" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>153</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="H4" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="H4" s="18">
+      <c r="I4" s="18">
         <f>(241822577+237201100)/(241822577+237201100+5856000+8368914)*100</f>
         <v>97.116076100458642</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>128</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>153</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="H5" s="18">
-        <f>100-H4</f>
+      <c r="I5" s="18">
+        <f>100-I4</f>
         <v>2.8839238995413581</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>128</v>
       </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>153</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="H6" s="10">
+      <c r="I6" s="10">
         <v>0</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>153</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="H7" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="H7" s="10">
+      <c r="I7" s="10">
         <v>0</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="15"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H8" s="6"/>
+      <c r="I8" s="15"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>159</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="H9" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="H9" s="11">
+      <c r="I9" s="11">
         <v>6.4777062142923141</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>128</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>159</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="H10" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="H10" s="11">
+      <c r="I10" s="11">
         <v>8.7567853491111922</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>128</v>
       </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
         <v>176</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>159</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="H11" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="H11" s="18">
+      <c r="I11" s="18">
         <v>59.671114354829328</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>128</v>
       </c>
-      <c r="J11" s="19" t="s">
+      <c r="K11" s="19" t="s">
         <v>177</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>159</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="H12" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="H12" s="18">
+      <c r="I12" s="18">
         <v>16.802918820320372</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>159</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="H13" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="H13" s="11">
+      <c r="I13" s="11">
         <v>7.4851294970113242</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>159</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="H14" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="H14" s="11">
+      <c r="I14" s="11">
         <v>0.80634576443547301</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F16" t="s">
         <v>121</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>130</v>
       </c>
-      <c r="H16" s="15">
+      <c r="I16" s="15">
         <v>80</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F17" t="s">
         <v>122</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>130</v>
       </c>
-      <c r="H17" s="15">
+      <c r="I17" s="15">
         <v>10</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F18" t="s">
         <v>123</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>130</v>
       </c>
-      <c r="H18" s="15">
+      <c r="I18" s="15">
         <v>10</v>
       </c>
-      <c r="I18" t="s">
+      <c r="J18" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C20" s="4"/>
+      <c r="H20" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="I20" s="26">
+        <v>0</v>
+      </c>
+      <c r="J20" s="9"/>
+      <c r="K20" s="9" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C21" s="4"/>
+      <c r="I21" s="18"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>153</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" t="s">
+        <v>184</v>
+      </c>
+      <c r="H22" t="s">
+        <v>183</v>
+      </c>
+      <c r="I22" s="18">
+        <f>74100</f>
+        <v>74100</v>
+      </c>
+      <c r="J22" t="s">
+        <v>194</v>
+      </c>
+      <c r="K22" t="s">
+        <v>188</v>
+      </c>
+      <c r="L22" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>153</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G23" t="s">
+        <v>192</v>
+      </c>
+      <c r="H23" t="s">
+        <v>183</v>
+      </c>
+      <c r="I23" s="11">
+        <f>3.9</f>
+        <v>3.9</v>
+      </c>
+      <c r="J23" t="s">
+        <v>194</v>
+      </c>
+      <c r="L23" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>153</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G24" t="s">
+        <v>185</v>
+      </c>
+      <c r="H24" t="s">
+        <v>183</v>
+      </c>
+      <c r="I24" s="11">
+        <f>3.9</f>
+        <v>3.9</v>
+      </c>
+      <c r="J24" t="s">
+        <v>194</v>
+      </c>
+      <c r="L24" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>153</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="G25" t="s">
+        <v>184</v>
+      </c>
+      <c r="H25" t="s">
+        <v>183</v>
+      </c>
+      <c r="I25" s="18">
+        <v>0</v>
+      </c>
+      <c r="J25" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>153</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="G26" t="s">
+        <v>193</v>
+      </c>
+      <c r="H26" t="s">
+        <v>183</v>
+      </c>
+      <c r="I26" s="23">
+        <f t="shared" ref="I26:I27" si="0">I23</f>
+        <v>3.9</v>
+      </c>
+      <c r="J26" t="s">
+        <v>194</v>
+      </c>
+      <c r="K26" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>153</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="G27" t="s">
+        <v>185</v>
+      </c>
+      <c r="H27" t="s">
+        <v>183</v>
+      </c>
+      <c r="I27" s="23">
+        <f t="shared" si="0"/>
+        <v>3.9</v>
+      </c>
+      <c r="J27" t="s">
+        <v>194</v>
+      </c>
+      <c r="K27" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>153</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="H28" t="s">
+        <v>183</v>
+      </c>
+      <c r="I28" s="18">
+        <v>0</v>
+      </c>
+      <c r="J28" t="s">
+        <v>194</v>
+      </c>
+      <c r="K28" s="15" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>153</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="H29" t="s">
+        <v>183</v>
+      </c>
+      <c r="I29" s="18">
+        <v>0</v>
+      </c>
+      <c r="J29" t="s">
+        <v>194</v>
+      </c>
+      <c r="K29" s="15"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C30" s="4"/>
+      <c r="I30" s="22"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>159</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="G31" t="s">
+        <v>184</v>
+      </c>
+      <c r="H31" t="s">
+        <v>183</v>
+      </c>
+      <c r="I31" s="18">
+        <v>73300</v>
+      </c>
+      <c r="J31" t="s">
+        <v>194</v>
+      </c>
+      <c r="K31" t="s">
+        <v>197</v>
+      </c>
+      <c r="L31" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>159</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="G32" t="s">
+        <v>192</v>
+      </c>
+      <c r="H32" t="s">
+        <v>183</v>
+      </c>
+      <c r="I32">
+        <v>10</v>
+      </c>
+      <c r="J32" t="s">
+        <v>194</v>
+      </c>
+      <c r="L32" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>159</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="G33" t="s">
+        <v>185</v>
+      </c>
+      <c r="H33" t="s">
+        <v>183</v>
+      </c>
+      <c r="I33">
+        <v>0.6</v>
+      </c>
+      <c r="J33" t="s">
+        <v>194</v>
+      </c>
+      <c r="L33" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>159</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="G34" t="s">
+        <v>184</v>
+      </c>
+      <c r="H34" t="s">
+        <v>183</v>
+      </c>
+      <c r="I34" s="18">
+        <v>56100</v>
+      </c>
+      <c r="J34" t="s">
+        <v>194</v>
+      </c>
+      <c r="K34" t="s">
+        <v>196</v>
+      </c>
+      <c r="L34" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>159</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="G35" t="s">
+        <v>192</v>
+      </c>
+      <c r="H35" t="s">
+        <v>183</v>
+      </c>
+      <c r="I35">
+        <v>5</v>
+      </c>
+      <c r="J35" t="s">
+        <v>194</v>
+      </c>
+      <c r="L35" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>159</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="G36" t="s">
+        <v>185</v>
+      </c>
+      <c r="H36" t="s">
+        <v>183</v>
+      </c>
+      <c r="I36">
+        <v>0.1</v>
+      </c>
+      <c r="J36" t="s">
+        <v>194</v>
+      </c>
+      <c r="L36" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>159</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="G37" t="s">
+        <v>184</v>
+      </c>
+      <c r="H37" t="s">
+        <v>183</v>
+      </c>
+      <c r="I37" s="18">
+        <v>0</v>
+      </c>
+      <c r="J37" t="s">
+        <v>194</v>
+      </c>
+      <c r="K37" t="s">
+        <v>195</v>
+      </c>
+      <c r="L37" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>159</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="G38" t="s">
+        <v>193</v>
+      </c>
+      <c r="H38" t="s">
+        <v>183</v>
+      </c>
+      <c r="I38" s="18">
+        <v>300</v>
+      </c>
+      <c r="J38" t="s">
+        <v>194</v>
+      </c>
+      <c r="L38" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>159</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="G39" t="s">
+        <v>185</v>
+      </c>
+      <c r="H39" t="s">
+        <v>183</v>
+      </c>
+      <c r="I39" s="18">
+        <v>4</v>
+      </c>
+      <c r="J39" t="s">
+        <v>194</v>
+      </c>
+      <c r="L39" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>159</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="H40" t="s">
+        <v>183</v>
+      </c>
+      <c r="I40" s="18">
+        <v>0</v>
+      </c>
+      <c r="J40" t="s">
+        <v>194</v>
+      </c>
+      <c r="K40" s="15"/>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>159</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="H41" t="s">
+        <v>183</v>
+      </c>
+      <c r="I41" s="18">
+        <v>0</v>
+      </c>
+      <c r="J41" t="s">
+        <v>194</v>
+      </c>
+      <c r="K41" s="15"/>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>159</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="H42" t="s">
+        <v>183</v>
+      </c>
+      <c r="I42" s="18">
+        <v>0</v>
+      </c>
+      <c r="J42" t="s">
+        <v>194</v>
+      </c>
+      <c r="K42" s="15"/>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C43" s="6"/>
+      <c r="I43" s="18"/>
+      <c r="K43" s="15"/>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A44" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="B44" s="15"/>
+      <c r="C44" s="24"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="15"/>
+      <c r="G44" s="15"/>
+      <c r="H44" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="I44" s="25">
+        <v>0</v>
+      </c>
+      <c r="K44" s="15"/>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I45" s="22"/>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
+      <c r="B46" s="1"/>
+      <c r="C46" s="1"/>
+      <c r="D46" s="1"/>
+      <c r="E46" s="1"/>
+      <c r="F46" s="1"/>
+      <c r="G46" s="1"/>
+      <c r="H46" s="1"/>
+      <c r="I46" s="1"/>
+      <c r="J46" s="1"/>
+      <c r="K46" s="1"/>
+      <c r="L46" s="1"/>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4" t="s">
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="3"/>
+      <c r="K47" s="3"/>
+      <c r="L47" s="3"/>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="H22">
+      <c r="I48">
         <v>10800</v>
       </c>
-      <c r="I22" t="s">
+      <c r="J48" t="s">
         <v>11</v>
       </c>
-      <c r="J22" s="4" t="s">
+      <c r="K48" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4" t="s">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B49" s="4"/>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4"/>
+      <c r="F49" s="4"/>
+      <c r="G49" s="4"/>
+      <c r="H49" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="H23">
+      <c r="I49">
         <v>5</v>
       </c>
-      <c r="I23" t="s">
+      <c r="J49" t="s">
         <v>13</v>
       </c>
-      <c r="J23" s="4" t="s">
+      <c r="K49" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="6" t="s">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4"/>
+      <c r="G50" s="4"/>
+      <c r="H50" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="H24">
+      <c r="I50">
         <v>2</v>
       </c>
-      <c r="I24" t="s">
+      <c r="J50" t="s">
         <v>126</v>
       </c>
-      <c r="J24" s="7"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4" t="s">
+      <c r="K50" s="7"/>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B51" s="4"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4"/>
+      <c r="G51" s="4"/>
+      <c r="H51" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H25">
+      <c r="I51">
         <v>0.2</v>
       </c>
-      <c r="I25" t="s">
+      <c r="J51" t="s">
         <v>15</v>
       </c>
-      <c r="J25" s="4" t="s">
+      <c r="K51" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4" t="s">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B52" s="4"/>
+      <c r="C52" s="4"/>
+      <c r="D52" s="4"/>
+      <c r="E52" s="4"/>
+      <c r="F52" s="4"/>
+      <c r="G52" s="4"/>
+      <c r="H52" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H26">
+      <c r="I52">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="I26" t="s">
+      <c r="J52" t="s">
         <v>17</v>
       </c>
-      <c r="J26" s="5" t="s">
+      <c r="K52" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="6" t="s">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B53" s="4"/>
+      <c r="C53" s="4"/>
+      <c r="D53" s="4"/>
+      <c r="E53" s="4"/>
+      <c r="F53" s="4"/>
+      <c r="G53" s="4"/>
+      <c r="H53" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="H27">
+      <c r="I53">
         <v>250</v>
       </c>
-      <c r="I27" t="s">
+      <c r="J53" t="s">
         <v>19</v>
       </c>
-      <c r="J27" s="5" t="s">
+      <c r="K53" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="20" t="s">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B54" s="4"/>
+      <c r="C54" s="4"/>
+      <c r="D54" s="4"/>
+      <c r="E54" s="4"/>
+      <c r="F54" s="4"/>
+      <c r="G54" s="4"/>
+      <c r="H54" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="H28" s="9">
+      <c r="I54" s="9">
         <v>1</v>
       </c>
-      <c r="I28" s="9"/>
-      <c r="J28" s="21" t="s">
+      <c r="J54" s="9"/>
+      <c r="K54" s="21" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="18" x14ac:dyDescent="0.35">
-      <c r="B29" s="4"/>
-      <c r="C29" s="4" t="s">
+    <row r="55" spans="1:16" ht="18" x14ac:dyDescent="0.35">
+      <c r="B55" s="4"/>
+      <c r="C55" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="6" t="s">
+      <c r="D55" s="4"/>
+      <c r="E55" s="4"/>
+      <c r="F55" s="4"/>
+      <c r="G55" s="4"/>
+      <c r="H55" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="H29">
+      <c r="I55">
         <v>0.26</v>
       </c>
-      <c r="J29" s="5" t="s">
+      <c r="K55" s="5" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="18" x14ac:dyDescent="0.35">
-      <c r="B30" s="4"/>
-      <c r="C30" s="4" t="s">
+    <row r="56" spans="1:16" ht="18" x14ac:dyDescent="0.35">
+      <c r="B56" s="4"/>
+      <c r="C56" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-      <c r="G30" s="6" t="s">
+      <c r="D56" s="4"/>
+      <c r="E56" s="4"/>
+      <c r="F56" s="4"/>
+      <c r="G56" s="4"/>
+      <c r="H56" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="H30">
+      <c r="I56">
         <v>0.26</v>
       </c>
-      <c r="J30" s="5" t="s">
+      <c r="K56" s="5" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="18" x14ac:dyDescent="0.35">
-      <c r="B31" s="4"/>
-      <c r="C31" s="4" t="s">
+    <row r="57" spans="1:16" ht="18" x14ac:dyDescent="0.35">
+      <c r="B57" s="4"/>
+      <c r="C57" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="6" t="s">
+      <c r="D57" s="4"/>
+      <c r="E57" s="4"/>
+      <c r="F57" s="4"/>
+      <c r="G57" s="4"/>
+      <c r="H57" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="H31">
+      <c r="I57">
         <v>0.45</v>
       </c>
-      <c r="J31" s="5" t="s">
+      <c r="K57" s="5" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="18" x14ac:dyDescent="0.35">
-      <c r="B32" s="4"/>
-      <c r="C32" s="6" t="s">
+    <row r="58" spans="1:16" ht="18" x14ac:dyDescent="0.35">
+      <c r="B58" s="4"/>
+      <c r="C58" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="D32" s="6"/>
-      <c r="E32" s="6"/>
-      <c r="F32" s="6"/>
-      <c r="G32" s="6" t="s">
+      <c r="D58" s="6"/>
+      <c r="E58" s="6"/>
+      <c r="F58" s="6"/>
+      <c r="G58" s="6"/>
+      <c r="H58" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="H32">
+      <c r="I58">
         <v>0.76</v>
       </c>
-      <c r="J32" s="5" t="s">
+      <c r="K58" s="5" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
-      <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="6" t="s">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B59" s="4"/>
+      <c r="C59" s="4"/>
+      <c r="D59" s="4"/>
+      <c r="E59" s="4"/>
+      <c r="F59" s="4"/>
+      <c r="G59" s="4"/>
+      <c r="H59" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="H33">
+      <c r="I59">
         <v>4</v>
       </c>
-      <c r="I33" t="s">
+      <c r="J59" t="s">
         <v>21</v>
       </c>
-      <c r="J33" s="7" t="s">
+      <c r="K59" s="7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A61" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
-      <c r="I35" s="2"/>
-      <c r="J35" s="2"/>
-      <c r="K35" s="2"/>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="G36" t="s">
+      <c r="B61" s="2"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2"/>
+      <c r="G61" s="2"/>
+      <c r="H61" s="2"/>
+      <c r="I61" s="2"/>
+      <c r="J61" s="2"/>
+      <c r="K61" s="2"/>
+      <c r="L61" s="2"/>
+    </row>
+    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="H62" t="s">
         <v>127</v>
       </c>
-      <c r="H36">
+      <c r="I62">
         <v>4</v>
       </c>
-      <c r="I36" t="s">
+      <c r="J62" t="s">
         <v>29</v>
       </c>
-      <c r="J36" t="s">
+      <c r="K62" t="s">
         <v>28</v>
       </c>
-      <c r="O36" s="6"/>
-    </row>
-    <row r="37" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="G37" t="s">
+      <c r="P62" s="6"/>
+    </row>
+    <row r="63" spans="1:16" ht="18" x14ac:dyDescent="0.35">
+      <c r="H63" t="s">
         <v>45</v>
       </c>
-      <c r="H37">
+      <c r="I63">
         <v>0.9</v>
       </c>
-      <c r="J37" t="s">
+      <c r="K63" t="s">
         <v>30</v>
       </c>
-      <c r="O37" s="6"/>
-    </row>
-    <row r="38" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="G38" t="s">
+      <c r="P63" s="6"/>
+    </row>
+    <row r="64" spans="1:16" ht="18" x14ac:dyDescent="0.35">
+      <c r="H64" t="s">
         <v>38</v>
       </c>
-      <c r="H38">
+      <c r="I64">
         <v>1.2250000000000001</v>
       </c>
-      <c r="I38" t="s">
+      <c r="J64" t="s">
         <v>32</v>
       </c>
-      <c r="J38" t="s">
+      <c r="K64" t="s">
         <v>31</v>
       </c>
-      <c r="O38" s="6"/>
-    </row>
-    <row r="39" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="G39" t="s">
+      <c r="P64" s="6"/>
+    </row>
+    <row r="65" spans="1:16" ht="18" x14ac:dyDescent="0.35">
+      <c r="H65" t="s">
         <v>39</v>
       </c>
-      <c r="H39">
+      <c r="I65">
         <v>0.1</v>
       </c>
-      <c r="J39" t="s">
+      <c r="K65" t="s">
         <v>33</v>
       </c>
-      <c r="O39" s="6"/>
-    </row>
-    <row r="40" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="G40" t="s">
+      <c r="P65" s="6"/>
+    </row>
+    <row r="66" spans="1:16" ht="18" x14ac:dyDescent="0.35">
+      <c r="H66" t="s">
         <v>40</v>
       </c>
-      <c r="H40">
+      <c r="I66">
         <v>0.01</v>
       </c>
-      <c r="J40" t="s">
+      <c r="K66" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="G41" t="s">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="H67" t="s">
         <v>41</v>
       </c>
-      <c r="H41">
+      <c r="I67">
         <v>0.2</v>
       </c>
-      <c r="J41" t="s">
+      <c r="K67" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="42" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="G42" t="s">
+    <row r="68" spans="1:16" ht="18" x14ac:dyDescent="0.35">
+      <c r="H68" t="s">
         <v>42</v>
       </c>
-      <c r="H42">
+      <c r="I68">
         <v>0.8</v>
       </c>
-      <c r="J42" t="s">
+      <c r="K68" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="43" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="G43" t="s">
+    <row r="69" spans="1:16" ht="18" x14ac:dyDescent="0.35">
+      <c r="H69" t="s">
         <v>43</v>
       </c>
-      <c r="H43">
+      <c r="I69">
         <v>55</v>
       </c>
-      <c r="J43" t="s">
+      <c r="K69" t="s">
         <v>37</v>
       </c>
-      <c r="N43" s="4"/>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A45" s="1" t="s">
+      <c r="O69" s="4"/>
+    </row>
+    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A71" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B45" s="8"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="8"/>
-      <c r="E45" s="8"/>
-      <c r="F45" s="8"/>
-      <c r="G45" s="8"/>
-      <c r="H45" s="8"/>
-      <c r="I45" s="8"/>
-      <c r="J45" s="8"/>
-      <c r="K45" s="8"/>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="G46" s="9" t="s">
+      <c r="B71" s="8"/>
+      <c r="C71" s="8"/>
+      <c r="D71" s="8"/>
+      <c r="E71" s="8"/>
+      <c r="F71" s="8"/>
+      <c r="G71" s="8"/>
+      <c r="H71" s="8"/>
+      <c r="I71" s="8"/>
+      <c r="J71" s="8"/>
+      <c r="K71" s="8"/>
+      <c r="L71" s="8"/>
+    </row>
+    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="H72" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="H46" s="9">
+      <c r="I72" s="9">
         <v>0</v>
       </c>
-      <c r="I46" s="9" t="s">
+      <c r="J72" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="J46" s="9"/>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="G47" s="9" t="s">
+      <c r="K72" s="9"/>
+    </row>
+    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="H73" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="H47" s="9">
+      <c r="I73" s="9">
         <v>0</v>
       </c>
-      <c r="I47" s="9" t="s">
+      <c r="J73" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="J47" s="9"/>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="G48" s="9" t="s">
+      <c r="K73" s="9"/>
+    </row>
+    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="H74" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="H48" s="9">
+      <c r="I74" s="9">
         <v>0</v>
       </c>
-      <c r="I48" s="9" t="s">
+      <c r="J74" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="J48" s="9"/>
-    </row>
-    <row r="49" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="G49" s="9" t="s">
+      <c r="K74" s="9"/>
+    </row>
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="H75" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="H49" s="9">
+      <c r="I75" s="9">
         <v>0</v>
       </c>
-      <c r="I49" s="9" t="s">
+      <c r="J75" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="J49" s="9"/>
-    </row>
-    <row r="50" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="G50" s="9" t="s">
+      <c r="K75" s="9"/>
+    </row>
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="H76" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="H50" s="9">
+      <c r="I76" s="9">
         <v>0</v>
       </c>
-      <c r="I50" s="9" t="s">
+      <c r="J76" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="J50" s="9"/>
-    </row>
-    <row r="51" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="G51" s="9" t="s">
+      <c r="K76" s="9"/>
+    </row>
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="H77" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="H51" s="9">
+      <c r="I77" s="9">
         <v>1</v>
       </c>
-      <c r="I51" s="9" t="s">
+      <c r="J77" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="J51" s="9" t="s">
+      <c r="K77" s="9" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="52" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="G52" s="9" t="s">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="H78" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="H52" s="9">
+      <c r="I78" s="9">
         <v>0</v>
       </c>
-      <c r="I52" s="9" t="s">
+      <c r="J78" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="J52" s="9"/>
-    </row>
-    <row r="53" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="G53" s="9" t="s">
+      <c r="K78" s="9"/>
+    </row>
+    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="H79" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="H53" s="9">
+      <c r="I79" s="9">
         <v>0</v>
       </c>
-      <c r="I53" s="9" t="s">
+      <c r="J79" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="J53" s="9"/>
-    </row>
-    <row r="54" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="G54" s="9" t="s">
+      <c r="K79" s="9"/>
+    </row>
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="H80" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="H54" s="9">
+      <c r="I80" s="9">
         <v>0</v>
       </c>
-      <c r="I54" s="9" t="s">
+      <c r="J80" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="J54" s="9"/>
-    </row>
-    <row r="55" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="G55" s="9" t="s">
+      <c r="K80" s="9"/>
+    </row>
+    <row r="81" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="H81" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="H55" s="9">
+      <c r="I81" s="9">
         <v>0</v>
       </c>
-      <c r="I55" s="9" t="s">
+      <c r="J81" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="J55" s="9"/>
-    </row>
-    <row r="56" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="G56" s="9"/>
-      <c r="H56" s="9"/>
-      <c r="I56" s="9"/>
-      <c r="J56" s="9"/>
-    </row>
-    <row r="57" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D57" t="s">
+      <c r="K81" s="9"/>
+    </row>
+    <row r="82" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="H82" s="9"/>
+      <c r="I82" s="9"/>
+      <c r="J82" s="9"/>
+      <c r="K82" s="9"/>
+    </row>
+    <row r="83" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D83" t="s">
         <v>60</v>
       </c>
-      <c r="G57" s="10" t="s">
+      <c r="H83" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="H57" s="10">
+      <c r="I83" s="10">
         <v>364</v>
       </c>
-      <c r="I57" s="10"/>
-      <c r="J57" s="10" t="s">
+      <c r="J83" s="10"/>
+      <c r="K83" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="K57" s="10"/>
-    </row>
-    <row r="58" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D58" t="s">
+      <c r="L83" s="10"/>
+    </row>
+    <row r="84" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D84" t="s">
         <v>60</v>
       </c>
-      <c r="G58" s="10" t="s">
+      <c r="H84" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="H58" s="10">
+      <c r="I84" s="10">
         <v>18.8</v>
       </c>
-      <c r="I58" s="10"/>
-      <c r="J58" s="10"/>
-      <c r="K58" s="10"/>
-    </row>
-    <row r="59" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D59" t="s">
+      <c r="J84" s="10"/>
+      <c r="K84" s="10"/>
+      <c r="L84" s="10"/>
+    </row>
+    <row r="85" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D85" t="s">
         <v>60</v>
       </c>
-      <c r="G59" s="10" t="s">
+      <c r="H85" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="H59" s="10">
+      <c r="I85" s="10">
         <v>0</v>
       </c>
-      <c r="I59" s="10"/>
-      <c r="J59" s="10"/>
-      <c r="K59" s="10"/>
-    </row>
-    <row r="60" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D60" t="s">
+      <c r="J85" s="10"/>
+      <c r="K85" s="10"/>
+      <c r="L85" s="10"/>
+    </row>
+    <row r="86" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D86" t="s">
         <v>60</v>
       </c>
-      <c r="G60" s="10" t="s">
+      <c r="H86" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="H60" s="10">
+      <c r="I86" s="10">
         <v>10</v>
       </c>
-      <c r="I60" s="10"/>
-      <c r="J60" s="10"/>
-      <c r="K60" s="10"/>
-    </row>
-    <row r="61" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D61" t="s">
+      <c r="J86" s="10"/>
+      <c r="K86" s="10"/>
+      <c r="L86" s="10"/>
+    </row>
+    <row r="87" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D87" t="s">
         <v>60</v>
       </c>
-      <c r="E61" t="s">
+      <c r="E87" t="s">
         <v>74</v>
       </c>
-      <c r="G61" s="10" t="s">
+      <c r="H87" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="H61" s="12">
+      <c r="I87" s="12">
         <v>1</v>
       </c>
-      <c r="I61" s="10"/>
-      <c r="J61" s="10"/>
-      <c r="K61" s="10"/>
-    </row>
-    <row r="62" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D62" t="s">
+      <c r="J87" s="10"/>
+      <c r="K87" s="10"/>
+      <c r="L87" s="10"/>
+    </row>
+    <row r="88" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D88" t="s">
         <v>60</v>
       </c>
-      <c r="E62" t="s">
+      <c r="E88" t="s">
         <v>73</v>
       </c>
-      <c r="G62" s="10" t="s">
+      <c r="H88" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="H62" s="10">
+      <c r="I88" s="10">
         <v>0.88</v>
       </c>
-      <c r="I62" s="10"/>
-      <c r="J62" s="10"/>
-      <c r="K62" s="10"/>
-    </row>
-    <row r="63" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D63" t="s">
+      <c r="J88" s="10"/>
+      <c r="K88" s="10"/>
+      <c r="L88" s="10"/>
+    </row>
+    <row r="89" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D89" t="s">
         <v>60</v>
       </c>
-      <c r="E63" t="s">
+      <c r="E89" t="s">
         <v>72</v>
       </c>
-      <c r="G63" s="10" t="s">
+      <c r="H89" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="H63" s="10">
+      <c r="I89" s="10">
         <v>0.78</v>
       </c>
-      <c r="I63" s="10"/>
-      <c r="J63" s="10"/>
-      <c r="K63" s="10"/>
-    </row>
-    <row r="64" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="G64" s="10"/>
-      <c r="H64" s="10"/>
-      <c r="I64" s="10"/>
-      <c r="J64" s="10"/>
-      <c r="K64" s="10"/>
-    </row>
-    <row r="65" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D65" t="s">
+      <c r="J89" s="10"/>
+      <c r="K89" s="10"/>
+      <c r="L89" s="10"/>
+    </row>
+    <row r="90" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="H90" s="10"/>
+      <c r="I90" s="10"/>
+      <c r="J90" s="10"/>
+      <c r="K90" s="10"/>
+      <c r="L90" s="10"/>
+    </row>
+    <row r="91" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D91" t="s">
         <v>63</v>
       </c>
-      <c r="G65" s="10" t="s">
+      <c r="H91" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="H65" s="10">
+      <c r="I91" s="10">
         <v>652</v>
       </c>
-      <c r="I65" s="10"/>
-      <c r="J65" s="10" t="s">
+      <c r="J91" s="10"/>
+      <c r="K91" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="K65" s="10"/>
-    </row>
-    <row r="66" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D66" t="s">
+      <c r="L91" s="10"/>
+    </row>
+    <row r="92" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D92" t="s">
         <v>63</v>
       </c>
-      <c r="G66" s="10" t="s">
+      <c r="H92" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="H66" s="10">
+      <c r="I92" s="10">
         <v>0</v>
       </c>
-      <c r="I66" s="10"/>
-      <c r="J66" s="10"/>
-      <c r="K66" s="10"/>
-    </row>
-    <row r="67" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D67" t="s">
+      <c r="J92" s="10"/>
+      <c r="K92" s="10"/>
+      <c r="L92" s="10"/>
+    </row>
+    <row r="93" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D93" t="s">
         <v>63</v>
       </c>
-      <c r="G67" s="10" t="s">
+      <c r="H93" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="H67" s="10">
+      <c r="I93" s="10">
         <v>5.0999999999999996</v>
       </c>
-      <c r="I67" s="10"/>
-      <c r="J67" s="10"/>
-      <c r="K67" s="10"/>
-    </row>
-    <row r="68" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D68" t="s">
+      <c r="J93" s="10"/>
+      <c r="K93" s="10"/>
+      <c r="L93" s="10"/>
+    </row>
+    <row r="94" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D94" t="s">
         <v>63</v>
       </c>
-      <c r="G68" s="10" t="s">
+      <c r="H94" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="H68" s="10">
+      <c r="I94" s="10">
         <v>20</v>
       </c>
-      <c r="I68" s="10"/>
-      <c r="J68" s="10"/>
-      <c r="K68" s="10"/>
-    </row>
-    <row r="69" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D69" t="s">
+      <c r="J94" s="10"/>
+      <c r="K94" s="10"/>
+      <c r="L94" s="10"/>
+    </row>
+    <row r="95" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D95" t="s">
         <v>63</v>
       </c>
-      <c r="E69" t="s">
+      <c r="E95" t="s">
         <v>74</v>
       </c>
-      <c r="G69" s="10" t="s">
+      <c r="H95" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="H69" s="12">
+      <c r="I95" s="12">
         <v>1</v>
       </c>
-      <c r="I69" s="10"/>
-      <c r="J69" s="10"/>
-      <c r="K69" s="10"/>
-    </row>
-    <row r="70" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D70" t="s">
+      <c r="J95" s="10"/>
+      <c r="K95" s="10"/>
+      <c r="L95" s="10"/>
+    </row>
+    <row r="96" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D96" t="s">
         <v>63</v>
       </c>
-      <c r="E70" t="s">
+      <c r="E96" t="s">
         <v>73</v>
       </c>
-      <c r="G70" s="10" t="s">
+      <c r="H96" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="H70" s="12">
+      <c r="I96" s="12">
         <v>0.7</v>
       </c>
-      <c r="I70" s="10"/>
-      <c r="J70" s="10"/>
-      <c r="K70" s="10"/>
-    </row>
-    <row r="71" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D71" t="s">
+      <c r="J96" s="10"/>
+      <c r="K96" s="10"/>
+      <c r="L96" s="10"/>
+    </row>
+    <row r="97" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D97" t="s">
         <v>63</v>
       </c>
-      <c r="E71" t="s">
+      <c r="E97" t="s">
         <v>72</v>
       </c>
-      <c r="G71" s="10" t="s">
+      <c r="H97" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="H71" s="10">
+      <c r="I97" s="10">
         <v>0.45</v>
       </c>
-      <c r="I71" s="10"/>
-      <c r="J71" s="10"/>
-      <c r="K71" s="10"/>
-    </row>
-    <row r="72" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="G72" s="10"/>
-      <c r="H72" s="10"/>
-      <c r="I72" s="10"/>
-      <c r="J72" s="10"/>
-      <c r="K72" s="10"/>
-    </row>
-    <row r="73" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D73" t="s">
+      <c r="J97" s="10"/>
+      <c r="K97" s="10"/>
+      <c r="L97" s="10"/>
+    </row>
+    <row r="98" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="H98" s="10"/>
+      <c r="I98" s="10"/>
+      <c r="J98" s="10"/>
+      <c r="K98" s="10"/>
+      <c r="L98" s="10"/>
+    </row>
+    <row r="99" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D99" t="s">
         <v>62</v>
       </c>
-      <c r="G73" s="10" t="s">
+      <c r="H99" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="H73" s="10">
+      <c r="I99" s="10">
         <v>46</v>
       </c>
-      <c r="I73" s="10"/>
-      <c r="J73" s="10" t="s">
+      <c r="J99" s="10"/>
+      <c r="K99" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="K73" s="10"/>
-    </row>
-    <row r="74" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D74" t="s">
+      <c r="L99" s="10"/>
+    </row>
+    <row r="100" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D100" t="s">
         <v>62</v>
       </c>
-      <c r="G74" s="10" t="s">
+      <c r="H100" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="H74" s="10">
+      <c r="I100" s="10">
         <v>2.8</v>
       </c>
-      <c r="I74" s="10"/>
-      <c r="J74" s="10"/>
-      <c r="K74" s="10"/>
-    </row>
-    <row r="75" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D75" t="s">
+      <c r="J100" s="10"/>
+      <c r="K100" s="10"/>
+      <c r="L100" s="10"/>
+    </row>
+    <row r="101" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D101" t="s">
         <v>62</v>
       </c>
-      <c r="G75" s="10" t="s">
+      <c r="H101" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="H75" s="10">
+      <c r="I101" s="10">
         <v>0</v>
       </c>
-      <c r="I75" s="10"/>
-      <c r="J75" s="10"/>
-      <c r="K75" s="10"/>
-    </row>
-    <row r="76" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D76" t="s">
+      <c r="J101" s="10"/>
+      <c r="K101" s="10"/>
+      <c r="L101" s="10"/>
+    </row>
+    <row r="102" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D102" t="s">
         <v>62</v>
       </c>
-      <c r="G76" s="10" t="s">
+      <c r="H102" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="H76" s="10">
+      <c r="I102" s="10">
         <v>5</v>
       </c>
-      <c r="I76" s="10"/>
-      <c r="J76" s="10"/>
-      <c r="K76" s="10"/>
-    </row>
-    <row r="77" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D77" t="s">
+      <c r="J102" s="10"/>
+      <c r="K102" s="10"/>
+      <c r="L102" s="10"/>
+    </row>
+    <row r="103" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D103" t="s">
         <v>62</v>
       </c>
-      <c r="E77" t="s">
+      <c r="E103" t="s">
         <v>74</v>
       </c>
-      <c r="G77" s="10" t="s">
+      <c r="H103" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="H77" s="12">
+      <c r="I103" s="12">
         <v>1</v>
       </c>
-      <c r="I77" s="10"/>
-      <c r="J77" s="10"/>
-      <c r="K77" s="10"/>
-    </row>
-    <row r="78" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D78" t="s">
+      <c r="J103" s="10"/>
+      <c r="K103" s="10"/>
+      <c r="L103" s="10"/>
+    </row>
+    <row r="104" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D104" t="s">
         <v>62</v>
       </c>
-      <c r="E78" t="s">
+      <c r="E104" t="s">
         <v>73</v>
       </c>
-      <c r="G78" s="10" t="s">
+      <c r="H104" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="H78" s="10">
+      <c r="I104" s="10">
         <v>0.85</v>
       </c>
-      <c r="I78" s="10"/>
-      <c r="J78" s="10"/>
-      <c r="K78" s="10"/>
-    </row>
-    <row r="79" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D79" t="s">
+      <c r="J104" s="10"/>
+      <c r="K104" s="10"/>
+      <c r="L104" s="10"/>
+    </row>
+    <row r="105" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D105" t="s">
         <v>62</v>
       </c>
-      <c r="E79" t="s">
+      <c r="E105" t="s">
         <v>72</v>
       </c>
-      <c r="G79" s="10" t="s">
+      <c r="H105" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="H79" s="10">
+      <c r="I105" s="10">
         <v>0.65</v>
       </c>
-      <c r="I79" s="10"/>
-      <c r="J79" s="10"/>
-      <c r="K79" s="10"/>
-    </row>
-    <row r="80" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="G80" s="10"/>
-      <c r="H80" s="10"/>
-      <c r="I80" s="10"/>
-      <c r="J80" s="10"/>
-      <c r="K80" s="10"/>
-    </row>
-    <row r="81" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="D81" t="s">
+      <c r="J105" s="10"/>
+      <c r="K105" s="10"/>
+      <c r="L105" s="10"/>
+    </row>
+    <row r="106" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="H106" s="10"/>
+      <c r="I106" s="10"/>
+      <c r="J106" s="10"/>
+      <c r="K106" s="10"/>
+      <c r="L106" s="10"/>
+    </row>
+    <row r="107" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D107" t="s">
         <v>65</v>
       </c>
-      <c r="G81" s="10" t="s">
+      <c r="H107" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="H81" s="12">
+      <c r="I107" s="12">
         <v>5.0999999999999996</v>
       </c>
-      <c r="I81" s="10"/>
-      <c r="J81" s="6" t="s">
+      <c r="J107" s="10"/>
+      <c r="K107" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="K81" s="4" t="s">
+      <c r="L107" s="4" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="82" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="D82" t="s">
+    <row r="108" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D108" t="s">
         <v>66</v>
       </c>
-      <c r="G82" s="10" t="s">
+      <c r="H108" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="H82" s="12">
+      <c r="I108" s="12">
         <v>7.1</v>
       </c>
-      <c r="I82" s="10"/>
-      <c r="J82" s="6" t="s">
+      <c r="J108" s="10"/>
+      <c r="K108" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="K82" s="4" t="s">
+      <c r="L108" s="4" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="83" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="G83" s="10"/>
-      <c r="H83" s="10"/>
-      <c r="I83" s="10"/>
-      <c r="J83" s="10"/>
-      <c r="K83" s="10"/>
-    </row>
-    <row r="84" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="D84" t="s">
+    <row r="109" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="H109" s="10"/>
+      <c r="I109" s="10"/>
+      <c r="J109" s="10"/>
+      <c r="K109" s="10"/>
+      <c r="L109" s="10"/>
+    </row>
+    <row r="110" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D110" t="s">
         <v>61</v>
       </c>
-      <c r="G84" s="10" t="s">
+      <c r="H110" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H84" s="12">
+      <c r="I110" s="12">
         <v>3.7353333333333332</v>
       </c>
-      <c r="I84" s="10"/>
-      <c r="J84" s="10" t="s">
+      <c r="J110" s="10"/>
+      <c r="K110" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="K84" s="6" t="s">
+      <c r="L110" s="6" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="85" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="D85" t="s">
+    <row r="111" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D111" t="s">
         <v>64</v>
       </c>
-      <c r="G85" s="10" t="s">
+      <c r="H111" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H85" s="11">
+      <c r="I111" s="11">
         <v>17.096931944444446</v>
       </c>
-      <c r="I85" s="10"/>
-      <c r="J85" s="6" t="s">
+      <c r="J111" s="10"/>
+      <c r="K111" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="K85" s="4" t="s">
+      <c r="L111" s="4" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="86" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="D86" t="s">
+    <row r="112" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="D112" t="s">
         <v>67</v>
       </c>
-      <c r="G86" s="10" t="s">
+      <c r="H112" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H86" s="12">
+      <c r="I112" s="12">
         <v>1.2451111111111113</v>
       </c>
-      <c r="I86" s="10"/>
-      <c r="J86" s="6" t="s">
+      <c r="J112" s="10"/>
+      <c r="K112" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="K86" s="10" t="s">
+      <c r="L112" s="10" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="87" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="D87" t="s">
+    <row r="113" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D113" t="s">
         <v>68</v>
       </c>
-      <c r="G87" s="10" t="s">
+      <c r="H113" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H87" s="12">
+      <c r="I113" s="12">
         <v>3.1127777777777781</v>
       </c>
-      <c r="I87" s="10"/>
-      <c r="J87" s="6" t="s">
+      <c r="J113" s="10"/>
+      <c r="K113" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="K87" s="10" t="s">
+      <c r="L113" s="10" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="88" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="D88" t="s">
+    <row r="114" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D114" t="s">
         <v>97</v>
       </c>
-      <c r="G88" s="10" t="s">
+      <c r="H114" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H88" s="12">
+      <c r="I114" s="12">
         <v>4.6691666666666665</v>
       </c>
-      <c r="I88" s="10"/>
-      <c r="J88" s="4" t="s">
+      <c r="J114" s="10"/>
+      <c r="K114" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="K88" s="10" t="s">
+      <c r="L114" s="10" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="89" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="D89" t="s">
+    <row r="115" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D115" t="s">
         <v>69</v>
       </c>
-      <c r="G89" s="10" t="s">
+      <c r="H115" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H89" s="12">
+      <c r="I115" s="12">
         <v>3.1127777777777781</v>
       </c>
-      <c r="I89" s="10"/>
-      <c r="J89" s="4" t="s">
+      <c r="J115" s="10"/>
+      <c r="K115" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="K89" s="6" t="s">
+      <c r="L115" s="6" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="90" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="D90" t="s">
+    <row r="116" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D116" t="s">
         <v>70</v>
       </c>
-      <c r="G90" s="10" t="s">
+      <c r="H116" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H90" s="11">
+      <c r="I116" s="11">
         <v>11.828555555555555</v>
       </c>
-      <c r="I90" s="10"/>
-      <c r="J90" s="4" t="s">
+      <c r="J116" s="10"/>
+      <c r="K116" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="K90" s="10" t="s">
+      <c r="L116" s="10" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="91" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="D91" t="s">
+    <row r="117" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D117" t="s">
         <v>100</v>
       </c>
-      <c r="G91" s="10" t="s">
+      <c r="H117" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H91" s="11">
+      <c r="I117" s="11">
         <v>26.302972222222223</v>
       </c>
-      <c r="I91" s="10"/>
-      <c r="J91" s="6" t="s">
+      <c r="J117" s="10"/>
+      <c r="K117" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="K91" s="10" t="s">
+      <c r="L117" s="10" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="92" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="D92" t="s">
+    <row r="118" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D118" t="s">
         <v>101</v>
       </c>
-      <c r="G92" s="10" t="s">
+      <c r="H118" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H92" s="11">
+      <c r="I118" s="11">
         <v>11.3</v>
       </c>
-      <c r="I92" s="10"/>
-      <c r="J92" s="6" t="s">
+      <c r="J118" s="10"/>
+      <c r="K118" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="K92" s="10" t="s">
+      <c r="L118" s="10" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="93" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="D93" t="s">
+    <row r="119" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D119" t="s">
         <v>102</v>
       </c>
-      <c r="G93" s="10" t="s">
+      <c r="H119" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H93" s="11">
+      <c r="I119" s="11">
         <v>23.278130416666666</v>
       </c>
-      <c r="I93" s="10"/>
-      <c r="J93" s="6" t="s">
+      <c r="J119" s="10"/>
+      <c r="K119" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="K93" s="10" t="s">
+      <c r="L119" s="10" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="94" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="D94" t="s">
+    <row r="120" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D120" t="s">
         <v>71</v>
       </c>
-      <c r="G94" s="10" t="s">
+      <c r="H120" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H94" s="10">
+      <c r="I120" s="10">
         <v>13.15</v>
       </c>
-      <c r="I94" s="10"/>
-      <c r="J94" s="10" t="s">
+      <c r="J120" s="10"/>
+      <c r="K120" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="K94" s="10" t="s">
+      <c r="L120" s="10" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="95" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="D95" t="s">
+    <row r="121" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D121" t="s">
         <v>71</v>
       </c>
-      <c r="G95" s="10" t="s">
+      <c r="H121" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="H95" s="10">
+      <c r="I121" s="10">
         <v>5.26</v>
       </c>
-      <c r="I95" s="10"/>
-      <c r="J95" s="10" t="s">
+      <c r="J121" s="10"/>
+      <c r="K121" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="K95" s="10" t="s">
+      <c r="L121" s="10" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="96" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B96" t="s">
+    <row r="122" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B122" t="s">
         <v>110</v>
       </c>
-      <c r="D96" t="s">
+      <c r="D122" t="s">
         <v>71</v>
       </c>
-      <c r="G96" s="10" t="s">
+      <c r="H122" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="H96" s="12">
+      <c r="I122" s="12">
         <v>1.7546281240590185</v>
       </c>
-      <c r="I96" s="10"/>
-      <c r="J96" s="10" t="s">
+      <c r="J122" s="10"/>
+      <c r="K122" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="K96" s="4" t="s">
+      <c r="L122" s="4" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B97" t="s">
+    <row r="123" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B123" t="s">
         <v>113</v>
       </c>
-      <c r="D97" t="s">
+      <c r="D123" t="s">
         <v>71</v>
       </c>
-      <c r="G97" s="10" t="s">
+      <c r="H123" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="H97" s="12">
+      <c r="I123" s="12">
         <v>5.1828516694033944</v>
       </c>
-      <c r="I97" s="10"/>
-      <c r="J97" s="6" t="s">
+      <c r="J123" s="10"/>
+      <c r="K123" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="K97" s="4" t="s">
+      <c r="L123" s="4" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B98" t="s">
+    <row r="124" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B124" t="s">
         <v>114</v>
       </c>
-      <c r="D98" t="s">
+      <c r="D124" t="s">
         <v>71</v>
       </c>
-      <c r="G98" s="10" t="s">
+      <c r="H124" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="H98" s="13">
+      <c r="I124" s="13">
         <v>4.0531064740502947</v>
       </c>
-      <c r="J98" s="6" t="s">
+      <c r="K124" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="K98" s="4" t="s">
+      <c r="L124" s="4" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B99" t="s">
+    <row r="125" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B125" t="s">
         <v>118</v>
       </c>
-      <c r="D99" t="s">
+      <c r="D125" t="s">
         <v>71</v>
       </c>
-      <c r="G99" s="10" t="s">
+      <c r="H125" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="H99" s="13">
+      <c r="I125" s="13">
         <v>4.3591310772039646</v>
       </c>
-      <c r="J99" s="6" t="s">
+      <c r="K125" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="K99" s="6" t="s">
+      <c r="L125" s="6" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="G100" s="10"/>
-      <c r="H100" s="13"/>
-      <c r="J100" s="6"/>
-      <c r="K100" s="6"/>
-    </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D101" t="s">
+    <row r="126" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="H126" s="10"/>
+      <c r="I126" s="13"/>
+      <c r="K126" s="6"/>
+      <c r="L126" s="6"/>
+    </row>
+    <row r="127" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D127" t="s">
         <v>120</v>
       </c>
-      <c r="G101" s="10" t="s">
+      <c r="H127" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H101" s="13">
+      <c r="I127" s="13">
         <v>14.6</v>
       </c>
-      <c r="J101" s="6"/>
-      <c r="K101" s="4" t="s">
+      <c r="K127" s="6"/>
+      <c r="L127" s="4" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D102" t="s">
+    <row r="128" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D128" t="s">
         <v>124</v>
       </c>
-      <c r="F102" t="s">
+      <c r="F128" t="s">
         <v>121</v>
       </c>
-      <c r="G102" s="10" t="s">
+      <c r="H128" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H102" s="13">
+      <c r="I128" s="13">
         <v>37.744765138888887</v>
       </c>
-      <c r="J102" s="6"/>
-      <c r="K102" s="6" t="s">
+      <c r="K128" s="6"/>
+      <c r="L128" s="6" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D103" t="s">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="D129" t="s">
         <v>124</v>
       </c>
-      <c r="F103" t="s">
+      <c r="F129" t="s">
         <v>122</v>
       </c>
-      <c r="G103" s="10" t="s">
+      <c r="H129" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H103" s="13">
+      <c r="I129" s="13">
         <v>50.107162083333336</v>
       </c>
-      <c r="J103" s="6"/>
-      <c r="K103" s="6" t="s">
+      <c r="K129" s="6"/>
+      <c r="L129" s="6" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D104" t="s">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="D130" t="s">
         <v>124</v>
       </c>
-      <c r="F104" t="s">
+      <c r="F130" t="s">
         <v>123</v>
       </c>
-      <c r="G104" s="10" t="s">
+      <c r="H130" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H104" s="13">
+      <c r="I130" s="13">
         <v>36.955675972222224</v>
       </c>
-      <c r="J104" s="6"/>
-      <c r="K104" s="6" t="s">
+      <c r="K130" s="6"/>
+      <c r="L130" s="6" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="G105" s="10"/>
-      <c r="H105" s="13"/>
-      <c r="J105" s="6"/>
-      <c r="K105" s="6"/>
-    </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D106" t="s">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H131" s="10"/>
+      <c r="I131" s="13"/>
+      <c r="K131" s="6"/>
+      <c r="L131" s="6"/>
+    </row>
+    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="D132" t="s">
         <v>131</v>
       </c>
-      <c r="G106" s="10" t="s">
+      <c r="H132" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="H106" s="13">
+      <c r="I132" s="13">
         <v>1.6176327916666666</v>
       </c>
-      <c r="J106" s="6" t="s">
+      <c r="K132" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="K106" s="4" t="s">
+      <c r="L132" s="4" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D107" t="s">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="D133" t="s">
         <v>132</v>
       </c>
-      <c r="G107" s="10" t="s">
+      <c r="H133" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="H107" s="13">
+      <c r="I133" s="13">
         <v>3.0774477499999997</v>
       </c>
-      <c r="J107" s="6" t="s">
+      <c r="K133" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="K107" s="4" t="s">
+      <c r="L133" s="4" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D108" t="s">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="D134" t="s">
         <v>133</v>
       </c>
-      <c r="G108" s="10" t="s">
+      <c r="H134" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="H108" s="13">
+      <c r="I134" s="13">
         <v>0.25</v>
       </c>
-      <c r="J108" s="6" t="s">
+      <c r="K134" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="K108" s="4" t="s">
+      <c r="L134" s="4" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A110" s="1" t="s">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A136" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B110" s="1"/>
-      <c r="C110" s="1"/>
-      <c r="D110" s="1"/>
-      <c r="E110" s="1"/>
-      <c r="F110" s="1"/>
-      <c r="G110" s="8"/>
-      <c r="H110" s="8"/>
-      <c r="I110" s="8"/>
-      <c r="J110" s="8"/>
-      <c r="K110" s="8"/>
-    </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="G111" s="9" t="s">
+      <c r="B136" s="1"/>
+      <c r="C136" s="1"/>
+      <c r="D136" s="1"/>
+      <c r="E136" s="1"/>
+      <c r="F136" s="1"/>
+      <c r="G136" s="1"/>
+      <c r="H136" s="8"/>
+      <c r="I136" s="8"/>
+      <c r="J136" s="8"/>
+      <c r="K136" s="8"/>
+      <c r="L136" s="8"/>
+    </row>
+    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H137" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="H111" s="9">
+      <c r="I137" s="9">
         <v>0</v>
       </c>
-      <c r="J111" s="9" t="s">
+      <c r="K137" s="9" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="G112" t="s">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H138" t="s">
         <v>49</v>
       </c>
-      <c r="H112" t="s">
+      <c r="I138" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A114" s="1" t="s">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A140" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="B114" s="1"/>
-      <c r="C114" s="1"/>
-      <c r="D114" s="1"/>
-      <c r="E114" s="1"/>
-      <c r="F114" s="1"/>
-      <c r="G114" s="8"/>
-      <c r="H114" s="8"/>
-      <c r="I114" s="8"/>
-      <c r="J114" s="8"/>
-      <c r="K114" s="8"/>
-    </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="G115" s="9" t="s">
+      <c r="B140" s="1"/>
+      <c r="C140" s="1"/>
+      <c r="D140" s="1"/>
+      <c r="E140" s="1"/>
+      <c r="F140" s="1"/>
+      <c r="G140" s="1"/>
+      <c r="H140" s="8"/>
+      <c r="I140" s="8"/>
+      <c r="J140" s="8"/>
+      <c r="K140" s="8"/>
+      <c r="L140" s="8"/>
+    </row>
+    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H141" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="H115" s="9">
+      <c r="I141" s="9">
         <v>0</v>
       </c>
-      <c r="I115" s="9" t="s">
+      <c r="J141" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="J115" s="9" t="s">
+      <c r="K141" s="9" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B116" t="s">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B142" t="s">
         <v>161</v>
       </c>
-      <c r="G116" t="s">
+      <c r="H142" t="s">
         <v>168</v>
       </c>
-      <c r="H116">
+      <c r="I142">
         <v>302</v>
       </c>
-      <c r="I116" t="s">
+      <c r="J142" t="s">
         <v>169</v>
       </c>
-      <c r="J116" t="s">
+      <c r="K142" t="s">
         <v>170</v>
       </c>
-      <c r="K116" t="s">
+      <c r="L142" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B117" t="s">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B143" t="s">
         <v>162</v>
       </c>
-      <c r="G117" t="s">
+      <c r="H143" t="s">
         <v>168</v>
       </c>
-      <c r="H117">
+      <c r="I143">
         <v>197</v>
       </c>
-      <c r="I117" t="s">
+      <c r="J143" t="s">
         <v>169</v>
       </c>
-      <c r="J117" t="s">
+      <c r="K143" t="s">
         <v>171</v>
       </c>
-      <c r="K117" t="s">
+      <c r="L143" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B118" t="s">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B144" t="s">
         <v>163</v>
       </c>
-      <c r="G118" t="s">
+      <c r="H144" t="s">
         <v>168</v>
       </c>
-      <c r="H118">
+      <c r="I144">
         <v>216</v>
       </c>
-      <c r="I118" t="s">
+      <c r="J144" t="s">
         <v>169</v>
       </c>
-      <c r="J118" t="s">
+      <c r="K144" t="s">
         <v>172</v>
       </c>
-      <c r="K118" t="s">
+      <c r="L144" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B119" t="s">
+    <row r="145" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B145" t="s">
         <v>164</v>
       </c>
-      <c r="G119" t="s">
+      <c r="H145" t="s">
         <v>168</v>
       </c>
-      <c r="H119">
+      <c r="I145">
         <v>216</v>
       </c>
-      <c r="I119" t="s">
+      <c r="J145" t="s">
         <v>169</v>
       </c>
-      <c r="J119" t="s">
+      <c r="K145" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B120" t="s">
+    <row r="146" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B146" t="s">
         <v>165</v>
       </c>
-      <c r="G120" t="s">
+      <c r="H146" t="s">
         <v>168</v>
       </c>
-      <c r="H120">
+      <c r="I146">
         <v>216</v>
       </c>
-      <c r="I120" t="s">
+      <c r="J146" t="s">
         <v>169</v>
       </c>
-      <c r="J120" t="s">
+      <c r="K146" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B121" t="s">
+    <row r="147" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B147" t="s">
         <v>166</v>
       </c>
-      <c r="G121" t="s">
+      <c r="H147" t="s">
         <v>168</v>
       </c>
-      <c r="H121">
+      <c r="I147">
         <v>216</v>
       </c>
-      <c r="I121" t="s">
+      <c r="J147" t="s">
         <v>169</v>
       </c>
-      <c r="J121" t="s">
+      <c r="K147" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B122" t="s">
+    <row r="148" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B148" t="s">
         <v>167</v>
       </c>
-      <c r="G122" t="s">
+      <c r="H148" t="s">
         <v>168</v>
       </c>
-      <c r="H122">
+      <c r="I148">
         <v>216</v>
       </c>
-      <c r="I122" t="s">
+      <c r="J148" t="s">
         <v>169</v>
       </c>
-      <c r="J122" t="s">
+      <c r="K148" t="s">
         <v>172</v>
       </c>
     </row>

</xml_diff>